<commit_message>
092425 - updated scores and skins for this week (9/22 week 21)
</commit_message>
<xml_diff>
--- a/public/results/2025/Week 21 Skins.xlsx
+++ b/public/results/2025/Week 21 Skins.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\CODE\golf-league-site\public\results\2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56943802-B1CC-4618-9677-A82E2CD9CB46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{56943802-B1CC-4618-9677-A82E2CD9CB46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D0B3174-EFE2-4F19-ABB1-36D3F29FDEAB}"/>
   <bookViews>
-    <workbookView xWindow="9690" yWindow="135" windowWidth="18975" windowHeight="10755" xr2:uid="{F705A57A-943D-4C93-A0B0-17476496A7BD}"/>
+    <workbookView xWindow="39945" yWindow="2655" windowWidth="30765" windowHeight="17115" xr2:uid="{F705A57A-943D-4C93-A0B0-17476496A7BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 21 Skins" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="31">
   <si>
     <t>Skins Won</t>
   </si>
@@ -93,6 +93,42 @@
   </si>
   <si>
     <t>John</t>
+  </si>
+  <si>
+    <t>Randy (.5)</t>
+  </si>
+  <si>
+    <t>Matt (.5)</t>
+  </si>
+  <si>
+    <t>Mark Y (1)</t>
+  </si>
+  <si>
+    <t>&lt;carry&gt;</t>
+  </si>
+  <si>
+    <t>Mike G (1)</t>
+  </si>
+  <si>
+    <t>Ryan (1)</t>
+  </si>
+  <si>
+    <t>Ryan (.5)</t>
+  </si>
+  <si>
+    <t>Aaron (.5)</t>
+  </si>
+  <si>
+    <t>Mark Y (.5)</t>
+  </si>
+  <si>
+    <t>Tony (.5)</t>
+  </si>
+  <si>
+    <t>Randy (1)</t>
+  </si>
+  <si>
+    <t>Mark Y (2)</t>
   </si>
 </sst>
 </file>
@@ -102,7 +138,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -148,13 +184,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -172,8 +201,23 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -198,6 +242,18 @@
         <bgColor rgb="FFD9E2F3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="26">
     <border>
@@ -543,7 +599,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -638,13 +694,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -668,10 +718,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -683,19 +745,28 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1033,33 +1104,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F8EC831-685C-42E6-9510-7BA05FCAF636}">
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.140625" style="4" customWidth="1"/>
     <col min="2" max="2" width="6.42578125" style="4" customWidth="1"/>
     <col min="3" max="11" width="8.7109375" style="4" customWidth="1"/>
     <col min="12" max="12" width="3.140625" style="4" customWidth="1"/>
-    <col min="13" max="13" width="5.42578125" style="41" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.42578125" style="39" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="6.28515625" style="4" customWidth="1"/>
     <col min="15" max="15" width="6.85546875" style="4" customWidth="1"/>
     <col min="16" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
       <c r="L1" s="14"/>
       <c r="M1" s="15" t="s">
         <v>0</v>
@@ -1103,10 +1174,10 @@
       <c r="K2" s="19">
         <v>9</v>
       </c>
-      <c r="L2" s="44" t="s">
-        <v>5</v>
-      </c>
-      <c r="M2" s="36"/>
+      <c r="L2" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="34"/>
       <c r="N2" s="6"/>
       <c r="O2" s="7"/>
     </row>
@@ -1142,8 +1213,8 @@
       <c r="K3" s="22">
         <v>5</v>
       </c>
-      <c r="L3" s="45"/>
-      <c r="M3" s="37"/>
+      <c r="L3" s="47"/>
+      <c r="M3" s="35"/>
       <c r="N3" s="8"/>
       <c r="O3" s="8"/>
     </row>
@@ -1179,8 +1250,8 @@
       <c r="K4" s="25">
         <v>2</v>
       </c>
-      <c r="L4" s="46"/>
-      <c r="M4" s="38"/>
+      <c r="L4" s="48"/>
+      <c r="M4" s="36"/>
       <c r="N4" s="11"/>
       <c r="O4" s="11"/>
     </row>
@@ -1191,35 +1262,35 @@
       <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="34">
-        <v>5</v>
-      </c>
-      <c r="D5" s="34">
+      <c r="C5" s="32">
+        <v>5</v>
+      </c>
+      <c r="D5" s="32">
         <v>8</v>
       </c>
-      <c r="E5" s="34">
-        <v>5</v>
-      </c>
-      <c r="F5" s="34">
-        <v>4</v>
-      </c>
-      <c r="G5" s="34">
-        <v>5</v>
-      </c>
-      <c r="H5" s="34">
-        <v>3</v>
-      </c>
-      <c r="I5" s="34">
-        <v>3</v>
-      </c>
-      <c r="J5" s="34">
-        <v>5</v>
-      </c>
-      <c r="K5" s="34">
+      <c r="E5" s="32">
+        <v>5</v>
+      </c>
+      <c r="F5" s="32">
+        <v>4</v>
+      </c>
+      <c r="G5" s="32">
+        <v>5</v>
+      </c>
+      <c r="H5" s="32">
+        <v>3</v>
+      </c>
+      <c r="I5" s="32">
+        <v>3</v>
+      </c>
+      <c r="J5" s="32">
+        <v>5</v>
+      </c>
+      <c r="K5" s="32">
         <v>5</v>
       </c>
       <c r="L5" s="27"/>
-      <c r="M5" s="39"/>
+      <c r="M5" s="37"/>
       <c r="N5" s="12"/>
       <c r="O5" s="6"/>
     </row>
@@ -1228,84 +1299,90 @@
       <c r="B6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="48">
-        <v>1</v>
-      </c>
-      <c r="D6" s="48">
-        <v>1</v>
-      </c>
-      <c r="E6" s="48">
-        <v>1</v>
-      </c>
-      <c r="F6" s="48">
-        <v>1</v>
-      </c>
-      <c r="G6" s="48">
-        <v>1</v>
-      </c>
-      <c r="H6" s="48">
-        <v>1</v>
-      </c>
-      <c r="I6" s="48">
-        <v>1</v>
-      </c>
-      <c r="J6" s="48">
-        <v>1</v>
-      </c>
-      <c r="K6" s="49">
+      <c r="C6" s="40">
+        <v>1</v>
+      </c>
+      <c r="D6" s="40">
+        <v>1</v>
+      </c>
+      <c r="E6" s="40">
+        <v>1</v>
+      </c>
+      <c r="F6" s="40">
+        <v>1</v>
+      </c>
+      <c r="G6" s="40">
+        <v>1</v>
+      </c>
+      <c r="H6" s="40">
+        <v>1</v>
+      </c>
+      <c r="I6" s="40">
+        <v>1</v>
+      </c>
+      <c r="J6" s="40">
+        <v>1</v>
+      </c>
+      <c r="K6" s="41">
         <v>1</v>
       </c>
       <c r="L6" s="29">
         <f>SUM(C6:K6)</f>
         <v>9</v>
       </c>
-      <c r="M6" s="40"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="8"/>
+      <c r="M6" s="38">
+        <v>1.5</v>
+      </c>
+      <c r="N6" s="9">
+        <v>7.5</v>
+      </c>
+      <c r="O6" s="8">
+        <v>7.5</v>
+      </c>
     </row>
     <row r="7" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="30"/>
       <c r="B7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="50">
+      <c r="C7" s="42">
         <f>C5-C6</f>
         <v>4</v>
       </c>
-      <c r="D7" s="50">
+      <c r="D7" s="42">
         <f t="shared" ref="D7:K7" si="0">D5-D6</f>
         <v>7</v>
       </c>
-      <c r="E7" s="50">
+      <c r="E7" s="42">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="F7" s="50">
+      <c r="F7" s="42">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G7" s="50">
+      <c r="G7" s="42">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="H7" s="50">
+      <c r="H7" s="49">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="I7" s="50">
+      <c r="I7" s="49">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="J7" s="50">
+      <c r="J7" s="42">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="K7" s="51">
+      <c r="K7" s="43">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="L7" s="31"/>
-      <c r="M7" s="35"/>
+      <c r="M7" s="33"/>
       <c r="N7" s="13"/>
       <c r="O7" s="10"/>
     </row>
@@ -1316,35 +1393,35 @@
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="34">
-        <v>4</v>
-      </c>
-      <c r="D8" s="34">
-        <v>6</v>
-      </c>
-      <c r="E8" s="34">
-        <v>5</v>
-      </c>
-      <c r="F8" s="34">
-        <v>6</v>
-      </c>
-      <c r="G8" s="34">
-        <v>6</v>
-      </c>
-      <c r="H8" s="34">
-        <v>4</v>
-      </c>
-      <c r="I8" s="34">
-        <v>4</v>
-      </c>
-      <c r="J8" s="34">
-        <v>6</v>
-      </c>
-      <c r="K8" s="34">
+      <c r="C8" s="32">
+        <v>4</v>
+      </c>
+      <c r="D8" s="32">
+        <v>6</v>
+      </c>
+      <c r="E8" s="32">
+        <v>5</v>
+      </c>
+      <c r="F8" s="32">
+        <v>6</v>
+      </c>
+      <c r="G8" s="32">
+        <v>6</v>
+      </c>
+      <c r="H8" s="32">
+        <v>4</v>
+      </c>
+      <c r="I8" s="32">
+        <v>4</v>
+      </c>
+      <c r="J8" s="32">
+        <v>6</v>
+      </c>
+      <c r="K8" s="32">
         <v>5</v>
       </c>
       <c r="L8" s="27"/>
-      <c r="M8" s="39"/>
+      <c r="M8" s="37"/>
       <c r="N8" s="12"/>
       <c r="O8" s="6"/>
     </row>
@@ -1353,84 +1430,90 @@
       <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="48">
-        <v>1</v>
-      </c>
-      <c r="D9" s="48">
-        <v>2</v>
-      </c>
-      <c r="E9" s="48">
-        <v>2</v>
-      </c>
-      <c r="F9" s="48">
-        <v>1</v>
-      </c>
-      <c r="G9" s="48">
-        <v>1</v>
-      </c>
-      <c r="H9" s="48">
-        <v>1</v>
-      </c>
-      <c r="I9" s="48">
-        <v>1</v>
-      </c>
-      <c r="J9" s="48">
-        <v>1</v>
-      </c>
-      <c r="K9" s="49">
+      <c r="C9" s="40">
+        <v>1</v>
+      </c>
+      <c r="D9" s="40">
+        <v>2</v>
+      </c>
+      <c r="E9" s="40">
+        <v>2</v>
+      </c>
+      <c r="F9" s="40">
+        <v>1</v>
+      </c>
+      <c r="G9" s="40">
+        <v>1</v>
+      </c>
+      <c r="H9" s="40">
+        <v>1</v>
+      </c>
+      <c r="I9" s="40">
+        <v>1</v>
+      </c>
+      <c r="J9" s="40">
+        <v>1</v>
+      </c>
+      <c r="K9" s="41">
         <v>2</v>
       </c>
       <c r="L9" s="29">
         <f>SUM(C9:K9)</f>
         <v>12</v>
       </c>
-      <c r="M9" s="40"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="8"/>
+      <c r="M9" s="38">
+        <v>1.5</v>
+      </c>
+      <c r="N9" s="9">
+        <v>7.5</v>
+      </c>
+      <c r="O9" s="8">
+        <v>7.5</v>
+      </c>
     </row>
     <row r="10" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="30"/>
       <c r="B10" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="50">
+      <c r="C10" s="49">
         <f>C8-C9</f>
         <v>3</v>
       </c>
-      <c r="D10" s="50">
+      <c r="D10" s="42">
         <f t="shared" ref="D10:K10" si="1">D8-D9</f>
         <v>4</v>
       </c>
-      <c r="E10" s="50">
+      <c r="E10" s="55">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="F10" s="50">
+      <c r="F10" s="42">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="G10" s="50">
+      <c r="G10" s="42">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="H10" s="50">
+      <c r="H10" s="42">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="I10" s="50">
+      <c r="I10" s="42">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="J10" s="50">
+      <c r="J10" s="42">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="K10" s="51">
+      <c r="K10" s="56">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="L10" s="31"/>
-      <c r="M10" s="35"/>
+      <c r="M10" s="33"/>
       <c r="N10" s="13"/>
       <c r="O10" s="10"/>
     </row>
@@ -1441,35 +1524,35 @@
       <c r="B11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="34">
-        <v>5</v>
-      </c>
-      <c r="D11" s="47">
-        <v>4</v>
-      </c>
-      <c r="E11" s="34">
-        <v>5</v>
-      </c>
-      <c r="F11" s="34">
-        <v>3</v>
-      </c>
-      <c r="G11" s="34">
-        <v>6</v>
-      </c>
-      <c r="H11" s="34">
-        <v>5</v>
-      </c>
-      <c r="I11" s="34">
-        <v>4</v>
-      </c>
-      <c r="J11" s="34">
-        <v>4</v>
-      </c>
-      <c r="K11" s="34">
+      <c r="C11" s="32">
+        <v>5</v>
+      </c>
+      <c r="D11" s="32">
+        <v>4</v>
+      </c>
+      <c r="E11" s="32">
+        <v>5</v>
+      </c>
+      <c r="F11" s="32">
+        <v>3</v>
+      </c>
+      <c r="G11" s="32">
+        <v>6</v>
+      </c>
+      <c r="H11" s="32">
+        <v>5</v>
+      </c>
+      <c r="I11" s="32">
+        <v>4</v>
+      </c>
+      <c r="J11" s="32">
+        <v>4</v>
+      </c>
+      <c r="K11" s="32">
         <v>10</v>
       </c>
       <c r="L11" s="29"/>
-      <c r="M11" s="39"/>
+      <c r="M11" s="37"/>
       <c r="N11" s="12"/>
       <c r="O11" s="6"/>
     </row>
@@ -1478,84 +1561,90 @@
       <c r="B12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="48">
-        <v>1</v>
-      </c>
-      <c r="D12" s="48">
-        <v>2</v>
-      </c>
-      <c r="E12" s="48">
-        <v>1</v>
-      </c>
-      <c r="F12" s="48">
-        <v>1</v>
-      </c>
-      <c r="G12" s="48">
-        <v>1</v>
-      </c>
-      <c r="H12" s="48">
-        <v>1</v>
-      </c>
-      <c r="I12" s="48">
-        <v>1</v>
-      </c>
-      <c r="J12" s="48">
-        <v>1</v>
-      </c>
-      <c r="K12" s="49">
+      <c r="C12" s="40">
+        <v>1</v>
+      </c>
+      <c r="D12" s="40">
+        <v>2</v>
+      </c>
+      <c r="E12" s="40">
+        <v>1</v>
+      </c>
+      <c r="F12" s="40">
+        <v>1</v>
+      </c>
+      <c r="G12" s="40">
+        <v>1</v>
+      </c>
+      <c r="H12" s="40">
+        <v>1</v>
+      </c>
+      <c r="I12" s="40">
+        <v>1</v>
+      </c>
+      <c r="J12" s="40">
+        <v>1</v>
+      </c>
+      <c r="K12" s="41">
         <v>2</v>
       </c>
       <c r="L12" s="29">
         <f>SUM(C12:K12)</f>
         <v>11</v>
       </c>
-      <c r="M12" s="40"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="8"/>
+      <c r="M12" s="38">
+        <v>3.5</v>
+      </c>
+      <c r="N12" s="9">
+        <v>17.5</v>
+      </c>
+      <c r="O12" s="8">
+        <v>18</v>
+      </c>
     </row>
     <row r="13" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="30"/>
       <c r="B13" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="50">
+      <c r="C13" s="42">
         <f>C11-C12</f>
         <v>4</v>
       </c>
-      <c r="D13" s="50">
+      <c r="D13" s="49">
         <f t="shared" ref="D13:K13" si="2">D11-D12</f>
         <v>2</v>
       </c>
-      <c r="E13" s="50">
+      <c r="E13" s="42">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="F13" s="50">
+      <c r="F13" s="49">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="G13" s="50">
+      <c r="G13" s="42">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="H13" s="50">
+      <c r="H13" s="42">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="I13" s="50">
+      <c r="I13" s="42">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="J13" s="50">
+      <c r="J13" s="49">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K13" s="50">
+      <c r="K13" s="42">
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="L13" s="31"/>
-      <c r="M13" s="35"/>
+      <c r="M13" s="33"/>
       <c r="N13" s="13"/>
       <c r="O13" s="10"/>
     </row>
@@ -1566,35 +1655,35 @@
       <c r="B14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="34">
-        <v>5</v>
-      </c>
-      <c r="D14" s="34">
-        <v>5</v>
-      </c>
-      <c r="E14" s="34">
-        <v>6</v>
-      </c>
-      <c r="F14" s="34">
-        <v>5</v>
-      </c>
-      <c r="G14" s="34">
-        <v>6</v>
-      </c>
-      <c r="H14" s="34">
+      <c r="C14" s="32">
+        <v>5</v>
+      </c>
+      <c r="D14" s="32">
+        <v>5</v>
+      </c>
+      <c r="E14" s="32">
+        <v>6</v>
+      </c>
+      <c r="F14" s="32">
+        <v>5</v>
+      </c>
+      <c r="G14" s="32">
+        <v>6</v>
+      </c>
+      <c r="H14" s="32">
         <v>7</v>
       </c>
-      <c r="I14" s="34">
-        <v>4</v>
-      </c>
-      <c r="J14" s="34">
-        <v>4</v>
-      </c>
-      <c r="K14" s="34">
+      <c r="I14" s="32">
+        <v>4</v>
+      </c>
+      <c r="J14" s="32">
+        <v>4</v>
+      </c>
+      <c r="K14" s="32">
         <v>6</v>
       </c>
       <c r="L14" s="29"/>
-      <c r="M14" s="39"/>
+      <c r="M14" s="37"/>
       <c r="N14" s="12"/>
       <c r="O14" s="6"/>
     </row>
@@ -1603,84 +1692,90 @@
       <c r="B15" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="48">
-        <v>1</v>
-      </c>
-      <c r="D15" s="48">
-        <v>2</v>
-      </c>
-      <c r="E15" s="48">
-        <v>2</v>
-      </c>
-      <c r="F15" s="48">
-        <v>1</v>
-      </c>
-      <c r="G15" s="48">
-        <v>1</v>
-      </c>
-      <c r="H15" s="48">
-        <v>1</v>
-      </c>
-      <c r="I15" s="48">
-        <v>1</v>
-      </c>
-      <c r="J15" s="48">
-        <v>1</v>
-      </c>
-      <c r="K15" s="49">
+      <c r="C15" s="40">
+        <v>1</v>
+      </c>
+      <c r="D15" s="40">
+        <v>2</v>
+      </c>
+      <c r="E15" s="40">
+        <v>2</v>
+      </c>
+      <c r="F15" s="40">
+        <v>1</v>
+      </c>
+      <c r="G15" s="40">
+        <v>1</v>
+      </c>
+      <c r="H15" s="40">
+        <v>1</v>
+      </c>
+      <c r="I15" s="40">
+        <v>1</v>
+      </c>
+      <c r="J15" s="40">
+        <v>1</v>
+      </c>
+      <c r="K15" s="41">
         <v>2</v>
       </c>
       <c r="L15" s="29">
         <f>SUM(C15:K15)</f>
         <v>12</v>
       </c>
-      <c r="M15" s="40"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="8"/>
+      <c r="M15" s="38">
+        <v>0.5</v>
+      </c>
+      <c r="N15" s="9">
+        <v>2.5</v>
+      </c>
+      <c r="O15" s="8">
+        <v>3</v>
+      </c>
     </row>
     <row r="16" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="30"/>
       <c r="B16" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="50">
+      <c r="C16" s="42">
         <f>C14-C15</f>
         <v>4</v>
       </c>
-      <c r="D16" s="50">
+      <c r="D16" s="42">
         <f t="shared" ref="D16:K16" si="3">D14-D15</f>
         <v>3</v>
       </c>
-      <c r="E16" s="50">
+      <c r="E16" s="42">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="F16" s="50">
+      <c r="F16" s="42">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="G16" s="50">
+      <c r="G16" s="42">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="H16" s="50">
+      <c r="H16" s="42">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="I16" s="50">
+      <c r="I16" s="42">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="J16" s="50">
+      <c r="J16" s="49">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="K16" s="50">
+      <c r="K16" s="42">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
       <c r="L16" s="31"/>
-      <c r="M16" s="35"/>
+      <c r="M16" s="33"/>
       <c r="N16" s="13"/>
       <c r="O16" s="10"/>
     </row>
@@ -1691,35 +1786,35 @@
       <c r="B17" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="34">
-        <v>6</v>
-      </c>
-      <c r="D17" s="34">
-        <v>6</v>
-      </c>
-      <c r="E17" s="34">
-        <v>5</v>
-      </c>
-      <c r="F17" s="34">
-        <v>5</v>
-      </c>
-      <c r="G17" s="34">
-        <v>4</v>
-      </c>
-      <c r="H17" s="34">
-        <v>5</v>
-      </c>
-      <c r="I17" s="34">
-        <v>4</v>
-      </c>
-      <c r="J17" s="34">
-        <v>6</v>
-      </c>
-      <c r="K17" s="34">
+      <c r="C17" s="32">
+        <v>6</v>
+      </c>
+      <c r="D17" s="32">
+        <v>6</v>
+      </c>
+      <c r="E17" s="32">
+        <v>5</v>
+      </c>
+      <c r="F17" s="32">
+        <v>5</v>
+      </c>
+      <c r="G17" s="32">
+        <v>4</v>
+      </c>
+      <c r="H17" s="32">
+        <v>5</v>
+      </c>
+      <c r="I17" s="32">
+        <v>4</v>
+      </c>
+      <c r="J17" s="32">
+        <v>6</v>
+      </c>
+      <c r="K17" s="32">
         <v>6</v>
       </c>
       <c r="L17" s="29"/>
-      <c r="M17" s="39"/>
+      <c r="M17" s="37"/>
       <c r="N17" s="12"/>
       <c r="O17" s="6"/>
     </row>
@@ -1728,84 +1823,90 @@
       <c r="B18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="48">
-        <v>2</v>
-      </c>
-      <c r="D18" s="48">
-        <v>2</v>
-      </c>
-      <c r="E18" s="48">
-        <v>2</v>
-      </c>
-      <c r="F18" s="48">
-        <v>1</v>
-      </c>
-      <c r="G18" s="48">
-        <v>2</v>
-      </c>
-      <c r="H18" s="48">
-        <v>1</v>
-      </c>
-      <c r="I18" s="48">
-        <v>1</v>
-      </c>
-      <c r="J18" s="48">
-        <v>2</v>
-      </c>
-      <c r="K18" s="49">
+      <c r="C18" s="40">
+        <v>2</v>
+      </c>
+      <c r="D18" s="40">
+        <v>2</v>
+      </c>
+      <c r="E18" s="40">
+        <v>2</v>
+      </c>
+      <c r="F18" s="40">
+        <v>1</v>
+      </c>
+      <c r="G18" s="40">
+        <v>2</v>
+      </c>
+      <c r="H18" s="40">
+        <v>1</v>
+      </c>
+      <c r="I18" s="40">
+        <v>1</v>
+      </c>
+      <c r="J18" s="40">
+        <v>2</v>
+      </c>
+      <c r="K18" s="41">
         <v>2</v>
       </c>
       <c r="L18" s="29">
         <f>SUM(C18:K18)</f>
         <v>15</v>
       </c>
-      <c r="M18" s="40"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="8"/>
+      <c r="M18" s="38">
+        <v>1</v>
+      </c>
+      <c r="N18" s="9">
+        <v>5</v>
+      </c>
+      <c r="O18" s="8">
+        <v>5</v>
+      </c>
     </row>
     <row r="19" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="30"/>
       <c r="B19" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="50">
+      <c r="C19" s="42">
         <f>C17-C18</f>
         <v>4</v>
       </c>
-      <c r="D19" s="50">
+      <c r="D19" s="42">
         <f t="shared" ref="D19:K19" si="4">D17-D18</f>
         <v>4</v>
       </c>
-      <c r="E19" s="50">
+      <c r="E19" s="55">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="F19" s="50">
+      <c r="F19" s="42">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="G19" s="50">
+      <c r="G19" s="49">
         <f t="shared" si="4"/>
         <v>2</v>
       </c>
-      <c r="H19" s="50">
+      <c r="H19" s="42">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="I19" s="50">
+      <c r="I19" s="42">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="J19" s="50">
+      <c r="J19" s="42">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="K19" s="50">
+      <c r="K19" s="42">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
       <c r="L19" s="31"/>
-      <c r="M19" s="35"/>
+      <c r="M19" s="33"/>
       <c r="N19" s="13"/>
       <c r="O19" s="10"/>
     </row>
@@ -1816,35 +1917,35 @@
       <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="34">
-        <v>5</v>
-      </c>
-      <c r="D20" s="34">
-        <v>5</v>
-      </c>
-      <c r="E20" s="34">
-        <v>4</v>
-      </c>
-      <c r="F20" s="34">
-        <v>5</v>
-      </c>
-      <c r="G20" s="34">
-        <v>4</v>
-      </c>
-      <c r="H20" s="34">
-        <v>4</v>
-      </c>
-      <c r="I20" s="34">
-        <v>4</v>
-      </c>
-      <c r="J20" s="34">
+      <c r="C20" s="32">
+        <v>5</v>
+      </c>
+      <c r="D20" s="32">
+        <v>5</v>
+      </c>
+      <c r="E20" s="32">
+        <v>4</v>
+      </c>
+      <c r="F20" s="32">
+        <v>5</v>
+      </c>
+      <c r="G20" s="32">
+        <v>4</v>
+      </c>
+      <c r="H20" s="32">
+        <v>4</v>
+      </c>
+      <c r="I20" s="32">
+        <v>4</v>
+      </c>
+      <c r="J20" s="32">
         <v>7</v>
       </c>
-      <c r="K20" s="34">
+      <c r="K20" s="32">
         <v>5</v>
       </c>
       <c r="L20" s="29"/>
-      <c r="M20" s="39"/>
+      <c r="M20" s="37"/>
       <c r="N20" s="12"/>
       <c r="O20" s="6"/>
     </row>
@@ -1853,34 +1954,34 @@
       <c r="B21" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="48">
-        <v>1</v>
-      </c>
-      <c r="D21" s="48">
-        <v>1</v>
-      </c>
-      <c r="E21" s="48">
-        <v>1</v>
-      </c>
-      <c r="F21" s="48"/>
-      <c r="G21" s="48">
-        <v>1</v>
-      </c>
-      <c r="H21" s="48">
-        <v>1</v>
-      </c>
-      <c r="I21" s="48"/>
-      <c r="J21" s="48">
-        <v>1</v>
-      </c>
-      <c r="K21" s="49">
+      <c r="C21" s="40">
+        <v>1</v>
+      </c>
+      <c r="D21" s="40">
+        <v>1</v>
+      </c>
+      <c r="E21" s="40">
+        <v>1</v>
+      </c>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40">
+        <v>1</v>
+      </c>
+      <c r="H21" s="40">
+        <v>1</v>
+      </c>
+      <c r="I21" s="40"/>
+      <c r="J21" s="40">
+        <v>1</v>
+      </c>
+      <c r="K21" s="41">
         <v>1</v>
       </c>
       <c r="L21" s="29">
         <f>SUM(C21:K21)</f>
         <v>7</v>
       </c>
-      <c r="M21" s="40"/>
+      <c r="M21" s="38"/>
       <c r="N21" s="9"/>
       <c r="O21" s="8"/>
     </row>
@@ -1889,44 +1990,44 @@
       <c r="B22" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="50">
+      <c r="C22" s="42">
         <f>C20-C21</f>
         <v>4</v>
       </c>
-      <c r="D22" s="50">
+      <c r="D22" s="42">
         <f t="shared" ref="D22:K22" si="5">D20-D21</f>
         <v>4</v>
       </c>
-      <c r="E22" s="50">
+      <c r="E22" s="55">
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="F22" s="50">
+      <c r="F22" s="42">
         <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="G22" s="50">
+      <c r="G22" s="42">
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="H22" s="50">
+      <c r="H22" s="42">
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="I22" s="50">
+      <c r="I22" s="42">
         <f t="shared" si="5"/>
         <v>4</v>
       </c>
-      <c r="J22" s="50">
+      <c r="J22" s="42">
         <f t="shared" si="5"/>
         <v>6</v>
       </c>
-      <c r="K22" s="50">
+      <c r="K22" s="42">
         <f t="shared" si="5"/>
         <v>4</v>
       </c>
       <c r="L22" s="31"/>
-      <c r="M22" s="35"/>
+      <c r="M22" s="33"/>
       <c r="N22" s="13"/>
       <c r="O22" s="10"/>
     </row>
@@ -1937,35 +2038,35 @@
       <c r="B23" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C23" s="34">
+      <c r="C23" s="32">
         <v>7</v>
       </c>
-      <c r="D23" s="34">
+      <c r="D23" s="32">
         <v>7</v>
       </c>
-      <c r="E23" s="34">
-        <v>5</v>
-      </c>
-      <c r="F23" s="34">
-        <v>4</v>
-      </c>
-      <c r="G23" s="34">
-        <v>5</v>
-      </c>
-      <c r="H23" s="34">
-        <v>5</v>
-      </c>
-      <c r="I23" s="34">
-        <v>3</v>
-      </c>
-      <c r="J23" s="34">
-        <v>5</v>
-      </c>
-      <c r="K23" s="34">
+      <c r="E23" s="32">
+        <v>5</v>
+      </c>
+      <c r="F23" s="32">
+        <v>4</v>
+      </c>
+      <c r="G23" s="32">
+        <v>5</v>
+      </c>
+      <c r="H23" s="32">
+        <v>5</v>
+      </c>
+      <c r="I23" s="32">
+        <v>3</v>
+      </c>
+      <c r="J23" s="32">
+        <v>5</v>
+      </c>
+      <c r="K23" s="32">
         <v>6</v>
       </c>
       <c r="L23" s="29"/>
-      <c r="M23" s="39"/>
+      <c r="M23" s="37"/>
       <c r="N23" s="12"/>
       <c r="O23" s="6"/>
     </row>
@@ -1974,84 +2075,90 @@
       <c r="B24" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="48">
-        <v>1</v>
-      </c>
-      <c r="D24" s="48">
-        <v>2</v>
-      </c>
-      <c r="E24" s="48">
-        <v>1</v>
-      </c>
-      <c r="F24" s="48">
-        <v>1</v>
-      </c>
-      <c r="G24" s="48">
-        <v>1</v>
-      </c>
-      <c r="H24" s="48">
-        <v>1</v>
-      </c>
-      <c r="I24" s="48">
-        <v>1</v>
-      </c>
-      <c r="J24" s="48">
-        <v>1</v>
-      </c>
-      <c r="K24" s="49">
+      <c r="C24" s="40">
+        <v>1</v>
+      </c>
+      <c r="D24" s="40">
+        <v>2</v>
+      </c>
+      <c r="E24" s="40">
+        <v>1</v>
+      </c>
+      <c r="F24" s="40">
+        <v>1</v>
+      </c>
+      <c r="G24" s="40">
+        <v>1</v>
+      </c>
+      <c r="H24" s="40">
+        <v>1</v>
+      </c>
+      <c r="I24" s="40">
+        <v>1</v>
+      </c>
+      <c r="J24" s="40">
+        <v>1</v>
+      </c>
+      <c r="K24" s="41">
         <v>1</v>
       </c>
       <c r="L24" s="29">
         <f>SUM(C24:K24)</f>
         <v>10</v>
       </c>
-      <c r="M24" s="40"/>
-      <c r="N24" s="9"/>
-      <c r="O24" s="8"/>
+      <c r="M24" s="38">
+        <v>0.5</v>
+      </c>
+      <c r="N24" s="9">
+        <v>2.5</v>
+      </c>
+      <c r="O24" s="8">
+        <v>3</v>
+      </c>
     </row>
     <row r="25" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="30"/>
       <c r="B25" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="50">
+      <c r="C25" s="42">
         <f>C23-C24</f>
         <v>6</v>
       </c>
-      <c r="D25" s="50">
+      <c r="D25" s="42">
         <f t="shared" ref="D25:K25" si="6">D23-D24</f>
         <v>5</v>
       </c>
-      <c r="E25" s="50">
+      <c r="E25" s="42">
         <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="F25" s="50">
+      <c r="F25" s="42">
         <f t="shared" si="6"/>
         <v>3</v>
       </c>
-      <c r="G25" s="50">
+      <c r="G25" s="42">
         <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="H25" s="50">
+      <c r="H25" s="42">
         <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="I25" s="50">
+      <c r="I25" s="49">
         <f t="shared" si="6"/>
         <v>2</v>
       </c>
-      <c r="J25" s="50">
+      <c r="J25" s="42">
         <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="K25" s="50">
+      <c r="K25" s="42">
         <f t="shared" si="6"/>
         <v>5</v>
       </c>
       <c r="L25" s="31"/>
-      <c r="M25" s="35"/>
+      <c r="M25" s="33"/>
       <c r="N25" s="13"/>
       <c r="O25" s="10"/>
     </row>
@@ -2062,35 +2169,35 @@
       <c r="B26" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C26" s="34">
-        <v>4</v>
-      </c>
-      <c r="D26" s="34">
-        <v>5</v>
-      </c>
-      <c r="E26" s="34">
-        <v>5</v>
-      </c>
-      <c r="F26" s="34">
-        <v>3</v>
-      </c>
-      <c r="G26" s="34">
-        <v>4</v>
-      </c>
-      <c r="H26" s="34">
-        <v>4</v>
-      </c>
-      <c r="I26" s="34">
-        <v>3</v>
-      </c>
-      <c r="J26" s="34">
-        <v>5</v>
-      </c>
-      <c r="K26" s="34">
+      <c r="C26" s="32">
+        <v>4</v>
+      </c>
+      <c r="D26" s="32">
+        <v>5</v>
+      </c>
+      <c r="E26" s="32">
+        <v>5</v>
+      </c>
+      <c r="F26" s="32">
+        <v>3</v>
+      </c>
+      <c r="G26" s="32">
+        <v>4</v>
+      </c>
+      <c r="H26" s="32">
+        <v>4</v>
+      </c>
+      <c r="I26" s="32">
+        <v>3</v>
+      </c>
+      <c r="J26" s="32">
+        <v>5</v>
+      </c>
+      <c r="K26" s="32">
         <v>5</v>
       </c>
       <c r="L26" s="29"/>
-      <c r="M26" s="39"/>
+      <c r="M26" s="37"/>
       <c r="N26" s="12"/>
       <c r="O26" s="6"/>
     </row>
@@ -2099,80 +2206,86 @@
       <c r="B27" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="48">
-        <v>1</v>
-      </c>
-      <c r="D27" s="48">
-        <v>1</v>
-      </c>
-      <c r="E27" s="48">
-        <v>1</v>
-      </c>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48">
-        <v>1</v>
-      </c>
-      <c r="H27" s="48">
-        <v>1</v>
-      </c>
-      <c r="I27" s="48"/>
-      <c r="J27" s="48">
-        <v>1</v>
-      </c>
-      <c r="K27" s="49">
+      <c r="C27" s="40">
+        <v>1</v>
+      </c>
+      <c r="D27" s="40">
+        <v>1</v>
+      </c>
+      <c r="E27" s="40">
+        <v>1</v>
+      </c>
+      <c r="F27" s="40"/>
+      <c r="G27" s="40">
+        <v>1</v>
+      </c>
+      <c r="H27" s="40">
+        <v>1</v>
+      </c>
+      <c r="I27" s="40"/>
+      <c r="J27" s="40">
+        <v>1</v>
+      </c>
+      <c r="K27" s="41">
         <v>1</v>
       </c>
       <c r="L27" s="29">
         <f>SUM(C27:K27)</f>
         <v>7</v>
       </c>
-      <c r="M27" s="40"/>
-      <c r="N27" s="9"/>
-      <c r="O27" s="8"/>
+      <c r="M27" s="38">
+        <v>0.5</v>
+      </c>
+      <c r="N27" s="9">
+        <v>2.5</v>
+      </c>
+      <c r="O27" s="8">
+        <v>3</v>
+      </c>
     </row>
     <row r="28" spans="1:15" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="30"/>
       <c r="B28" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C28" s="50">
+      <c r="C28" s="49">
         <f>C26-C27</f>
         <v>3</v>
       </c>
-      <c r="D28" s="50">
+      <c r="D28" s="42">
         <f t="shared" ref="D28:K28" si="7">D26-D27</f>
         <v>4</v>
       </c>
-      <c r="E28" s="50">
+      <c r="E28" s="42">
         <f t="shared" si="7"/>
         <v>4</v>
       </c>
-      <c r="F28" s="50">
+      <c r="F28" s="42">
         <f t="shared" si="7"/>
         <v>3</v>
       </c>
-      <c r="G28" s="50">
+      <c r="G28" s="42">
         <f t="shared" si="7"/>
         <v>3</v>
       </c>
-      <c r="H28" s="50">
+      <c r="H28" s="42">
         <f t="shared" si="7"/>
         <v>3</v>
       </c>
-      <c r="I28" s="50">
+      <c r="I28" s="42">
         <f t="shared" si="7"/>
         <v>3</v>
       </c>
-      <c r="J28" s="50">
+      <c r="J28" s="42">
         <f t="shared" si="7"/>
         <v>4</v>
       </c>
-      <c r="K28" s="50">
+      <c r="K28" s="42">
         <f t="shared" si="7"/>
         <v>4</v>
       </c>
       <c r="L28" s="31"/>
-      <c r="M28" s="35"/>
+      <c r="M28" s="33"/>
       <c r="N28" s="13"/>
       <c r="O28" s="10"/>
     </row>
@@ -2183,35 +2296,35 @@
       <c r="B29" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C29" s="34">
-        <v>6</v>
-      </c>
-      <c r="D29" s="34">
-        <v>6</v>
-      </c>
-      <c r="E29" s="34">
-        <v>6</v>
-      </c>
-      <c r="F29" s="34">
-        <v>4</v>
-      </c>
-      <c r="G29" s="34">
-        <v>5</v>
-      </c>
-      <c r="H29" s="34">
+      <c r="C29" s="32">
+        <v>6</v>
+      </c>
+      <c r="D29" s="32">
+        <v>6</v>
+      </c>
+      <c r="E29" s="32">
+        <v>6</v>
+      </c>
+      <c r="F29" s="32">
+        <v>4</v>
+      </c>
+      <c r="G29" s="32">
+        <v>5</v>
+      </c>
+      <c r="H29" s="32">
         <v>7</v>
       </c>
-      <c r="I29" s="34">
-        <v>6</v>
-      </c>
-      <c r="J29" s="34">
-        <v>6</v>
-      </c>
-      <c r="K29" s="34">
+      <c r="I29" s="32">
+        <v>6</v>
+      </c>
+      <c r="J29" s="32">
+        <v>6</v>
+      </c>
+      <c r="K29" s="32">
         <v>6</v>
       </c>
       <c r="L29" s="29"/>
-      <c r="M29" s="39"/>
+      <c r="M29" s="37"/>
       <c r="N29" s="12"/>
       <c r="O29" s="6"/>
     </row>
@@ -2220,38 +2333,38 @@
       <c r="B30" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="48">
-        <v>2</v>
-      </c>
-      <c r="D30" s="48">
-        <v>2</v>
-      </c>
-      <c r="E30" s="48">
-        <v>2</v>
-      </c>
-      <c r="F30" s="48">
-        <v>1</v>
-      </c>
-      <c r="G30" s="48">
-        <v>2</v>
-      </c>
-      <c r="H30" s="48">
-        <v>1</v>
-      </c>
-      <c r="I30" s="48">
-        <v>1</v>
-      </c>
-      <c r="J30" s="48">
-        <v>1</v>
-      </c>
-      <c r="K30" s="49">
+      <c r="C30" s="40">
+        <v>2</v>
+      </c>
+      <c r="D30" s="40">
+        <v>2</v>
+      </c>
+      <c r="E30" s="40">
+        <v>2</v>
+      </c>
+      <c r="F30" s="40">
+        <v>1</v>
+      </c>
+      <c r="G30" s="40">
+        <v>2</v>
+      </c>
+      <c r="H30" s="40">
+        <v>1</v>
+      </c>
+      <c r="I30" s="40">
+        <v>1</v>
+      </c>
+      <c r="J30" s="40">
+        <v>1</v>
+      </c>
+      <c r="K30" s="41">
         <v>2</v>
       </c>
       <c r="L30" s="29">
         <f>SUM(C30:K30)</f>
         <v>14</v>
       </c>
-      <c r="M30" s="40"/>
+      <c r="M30" s="38"/>
       <c r="N30" s="9"/>
       <c r="O30" s="8"/>
     </row>
@@ -2260,60 +2373,113 @@
       <c r="B31" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C31" s="50">
+      <c r="C31" s="42">
         <f>C29-C30</f>
         <v>4</v>
       </c>
-      <c r="D31" s="50">
+      <c r="D31" s="42">
         <f t="shared" ref="D31:K31" si="8">D29-D30</f>
         <v>4</v>
       </c>
-      <c r="E31" s="50">
+      <c r="E31" s="42">
         <f t="shared" si="8"/>
         <v>4</v>
       </c>
-      <c r="F31" s="50">
+      <c r="F31" s="42">
         <f t="shared" si="8"/>
         <v>3</v>
       </c>
-      <c r="G31" s="50">
+      <c r="G31" s="42">
         <f t="shared" si="8"/>
         <v>3</v>
       </c>
-      <c r="H31" s="50">
+      <c r="H31" s="42">
         <f t="shared" si="8"/>
         <v>6</v>
       </c>
-      <c r="I31" s="50">
+      <c r="I31" s="42">
         <f t="shared" si="8"/>
         <v>5</v>
       </c>
-      <c r="J31" s="50">
+      <c r="J31" s="42">
         <f t="shared" si="8"/>
         <v>5</v>
       </c>
-      <c r="K31" s="50">
+      <c r="K31" s="42">
         <f t="shared" si="8"/>
         <v>4</v>
       </c>
       <c r="L31" s="31"/>
-      <c r="M31" s="35"/>
+      <c r="M31" s="33"/>
       <c r="N31" s="13"/>
       <c r="O31" s="10"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="M32" s="41">
-        <f>SUM(M7:M31)</f>
-        <v>0</v>
-      </c>
-      <c r="N32" s="33">
-        <f>SUM(N7:N31)</f>
-        <v>0</v>
-      </c>
-      <c r="O32" s="32">
-        <f>SUM(O7:O31)</f>
-        <v>0</v>
-      </c>
+      <c r="A32" s="50"/>
+      <c r="B32" s="50"/>
+      <c r="C32" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="E32" s="54" t="s">
+        <v>22</v>
+      </c>
+      <c r="F32" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="G32" s="50" t="s">
+        <v>23</v>
+      </c>
+      <c r="H32" s="50" t="s">
+        <v>24</v>
+      </c>
+      <c r="I32" s="50" t="s">
+        <v>25</v>
+      </c>
+      <c r="J32" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="K32" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="L32" s="50"/>
+      <c r="M32" s="51">
+        <f>SUM(M5:M31)</f>
+        <v>9</v>
+      </c>
+      <c r="N32" s="52">
+        <f>SUM(N5:N31)</f>
+        <v>45</v>
+      </c>
+      <c r="O32" s="53">
+        <f>SUM(O6:O31)</f>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" s="50"/>
+      <c r="B33" s="50"/>
+      <c r="C33" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="50"/>
+      <c r="E33" s="50"/>
+      <c r="F33" s="50"/>
+      <c r="G33" s="50"/>
+      <c r="H33" s="50"/>
+      <c r="I33" s="50" t="s">
+        <v>26</v>
+      </c>
+      <c r="J33" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="K33" s="50"/>
+      <c r="L33" s="50"/>
+      <c r="M33" s="51"/>
+      <c r="N33" s="50"/>
+      <c r="O33" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>